<commit_message>
removal of unneeded files
</commit_message>
<xml_diff>
--- a/server/exports/weekly-summary.xlsx
+++ b/server/exports/weekly-summary.xlsx
@@ -16,7 +16,7 @@
     <t>Summary Report</t>
   </si>
   <si>
-    <t>2026-06-25 to 2026-06-30</t>
+    <t>2026-06-27 to 2026-07-02</t>
   </si>
   <si>
     <t>Reporter</t>
@@ -31,10 +31,10 @@
     <t>Amene Terhemen</t>
   </si>
   <si>
-    <t>Adeeko Bridget</t>
-  </si>
-  <si>
-    <t>Ikpuri Eyoanwan</t>
+    <t>Adeeko Bridget Olufunmilola</t>
+  </si>
+  <si>
+    <t>Ikpuri Eyoanwan Olaitan</t>
   </si>
 </sst>
 </file>
@@ -471,10 +471,10 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C5">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -482,7 +482,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C6">
         <v>0</v>

</xml_diff>

<commit_message>
changed doc url for web access
</commit_message>
<xml_diff>
--- a/server/exports/weekly-summary.xlsx
+++ b/server/exports/weekly-summary.xlsx
@@ -16,7 +16,7 @@
     <t>Summary Report</t>
   </si>
   <si>
-    <t>2026-06-27 to 2026-07-02</t>
+    <t>2026-06-27 to 2026-07-03</t>
   </si>
   <si>
     <t>Reporter</t>
@@ -28,7 +28,7 @@
     <t>Interventions</t>
   </si>
   <si>
-    <t>Amene Terhemen</t>
+    <t>Amene Ter'Hemen</t>
   </si>
   <si>
     <t>Adeeko Bridget Olufunmilola</t>

</xml_diff>

<commit_message>
changes to dashsidebar UI
</commit_message>
<xml_diff>
--- a/server/exports/weekly-summary.xlsx
+++ b/server/exports/weekly-summary.xlsx
@@ -11,12 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>Summary Report</t>
   </si>
   <si>
-    <t>2026-06-27 to 2026-07-03</t>
+    <t>2026-07-04 to 2026-07-06</t>
   </si>
   <si>
     <t>Reporter</t>
@@ -28,13 +28,10 @@
     <t>Interventions</t>
   </si>
   <si>
-    <t>Amene Ter'Hemen</t>
-  </si>
-  <si>
-    <t>Adeeko Bridget Olufunmilola</t>
-  </si>
-  <si>
-    <t>Ikpuri Eyoanwan Olaitan</t>
+    <t>OGWU Joshua Ugbede</t>
+  </si>
+  <si>
+    <t>UGWUOKE Rachael Nneoma</t>
   </si>
 </sst>
 </file>
@@ -433,7 +430,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -474,7 +471,7 @@
         <v>1</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -482,20 +479,9 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7">
-        <v>1</v>
-      </c>
-      <c r="C7">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fixed outOfStock saving error
</commit_message>
<xml_diff>
--- a/server/exports/weekly-summary.xlsx
+++ b/server/exports/weekly-summary.xlsx
@@ -11,12 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>Summary Report</t>
   </si>
   <si>
-    <t>2026-07-04 to 2026-07-06</t>
+    <t>2026-07-05 to 2026-07-11</t>
   </si>
   <si>
     <t>Reporter</t>
@@ -32,6 +32,78 @@
   </si>
   <si>
     <t>UGWUOKE Rachael Nneoma</t>
+  </si>
+  <si>
+    <t>EWERE Godswork Odion</t>
+  </si>
+  <si>
+    <t>LAAGO Blessing Kabari</t>
+  </si>
+  <si>
+    <t>BABAJIDE Oyetunji</t>
+  </si>
+  <si>
+    <t>IKUKOYI Dayo Sunday</t>
+  </si>
+  <si>
+    <t>OMBULE Daniel Blessing</t>
+  </si>
+  <si>
+    <t>OMOYOMI Oluwatosin Clinton</t>
+  </si>
+  <si>
+    <t>SAMUEL Onyedika Samuel</t>
+  </si>
+  <si>
+    <t>ATITI Joy Oghenerukevwe Tekena</t>
+  </si>
+  <si>
+    <t>TAIWO Temitope Joseph</t>
+  </si>
+  <si>
+    <t>ADEOSUN Taiwo</t>
+  </si>
+  <si>
+    <t>OGHENEWOGAGA Michael Fejiro</t>
+  </si>
+  <si>
+    <t>OLAYINKA Olalekan Jacob</t>
+  </si>
+  <si>
+    <t>CHUKWUNURU Christian Chidoziem</t>
+  </si>
+  <si>
+    <t>ABIONA Damilola Peace</t>
+  </si>
+  <si>
+    <t>SOLOMON Ajibade Favour</t>
+  </si>
+  <si>
+    <t>FATOBA Ruth Tofunmi</t>
+  </si>
+  <si>
+    <t>OKEOWO Toluwani Elizabeth</t>
+  </si>
+  <si>
+    <t>UGOBI Michael Chidiebere</t>
+  </si>
+  <si>
+    <t>AKINLEYE Onaopemipo Glory</t>
+  </si>
+  <si>
+    <t>ANUKAM Chinazaekpere Peace</t>
+  </si>
+  <si>
+    <t>FABUSUYI Yetunde Hope</t>
+  </si>
+  <si>
+    <t>APATA Victor Paul</t>
+  </si>
+  <si>
+    <t>AFOLABI Bukola Adejoke</t>
+  </si>
+  <si>
+    <t>AMENE Ter'Hemen</t>
   </si>
 </sst>
 </file>
@@ -430,7 +502,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -468,7 +540,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -479,10 +551,274 @@
         <v>6</v>
       </c>
       <c r="B6">
+        <v>5</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7">
+        <v>4</v>
+      </c>
+      <c r="C7">
         <v>1</v>
       </c>
-      <c r="C6">
-        <v>0</v>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8">
+        <v>6</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9">
+        <v>3</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11">
+        <v>4</v>
+      </c>
+      <c r="C11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12">
+        <v>2</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13">
+        <v>4</v>
+      </c>
+      <c r="C13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14">
+        <v>4</v>
+      </c>
+      <c r="C14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>15</v>
+      </c>
+      <c r="B15">
+        <v>4</v>
+      </c>
+      <c r="C15">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>16</v>
+      </c>
+      <c r="B16">
+        <v>5</v>
+      </c>
+      <c r="C16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+      <c r="C17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>18</v>
+      </c>
+      <c r="B18">
+        <v>3</v>
+      </c>
+      <c r="C18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>19</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>20</v>
+      </c>
+      <c r="B20">
+        <v>3</v>
+      </c>
+      <c r="C20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>21</v>
+      </c>
+      <c r="B21">
+        <v>4</v>
+      </c>
+      <c r="C21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>22</v>
+      </c>
+      <c r="B22">
+        <v>4</v>
+      </c>
+      <c r="C22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>23</v>
+      </c>
+      <c r="B23">
+        <v>2</v>
+      </c>
+      <c r="C23">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>24</v>
+      </c>
+      <c r="B24">
+        <v>2</v>
+      </c>
+      <c r="C24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>25</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>26</v>
+      </c>
+      <c r="B26">
+        <v>3</v>
+      </c>
+      <c r="C26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>27</v>
+      </c>
+      <c r="B27">
+        <v>3</v>
+      </c>
+      <c r="C27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>28</v>
+      </c>
+      <c r="B28">
+        <v>1</v>
+      </c>
+      <c r="C28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>29</v>
+      </c>
+      <c r="B29">
+        <v>1</v>
+      </c>
+      <c r="C29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>30</v>
+      </c>
+      <c r="B30">
+        <v>1</v>
+      </c>
+      <c r="C30">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
adjusted report generation to include those with zero reports
</commit_message>
<xml_diff>
--- a/server/exports/weekly-summary.xlsx
+++ b/server/exports/weekly-summary.xlsx
@@ -11,12 +11,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
   <si>
     <t>Summary Report</t>
   </si>
   <si>
-    <t>2026-07-05 to 2026-07-11</t>
+    <t>2026-08-16 to 2026-08-22</t>
   </si>
   <si>
     <t>Reporter</t>
@@ -28,82 +28,103 @@
     <t>Interventions</t>
   </si>
   <si>
+    <t>AMENE Ter'Hemen</t>
+  </si>
+  <si>
+    <t>CHUKWUNURU Christian Chidoziem</t>
+  </si>
+  <si>
+    <t>OLADUNNI Amos Abimbola</t>
+  </si>
+  <si>
+    <t>DABANG Naanchin Emmanuel</t>
+  </si>
+  <si>
+    <t>OMBULE Daniel Blessing</t>
+  </si>
+  <si>
+    <t>ANUKAM Chinazaekpere Peace</t>
+  </si>
+  <si>
+    <t>OKEOWO Toluwani Elizabeth</t>
+  </si>
+  <si>
     <t>OGWU Joshua Ugbede</t>
   </si>
   <si>
+    <t>FATOBA Ruth Tofunmi</t>
+  </si>
+  <si>
+    <t>OGHENEWOGAGA Michael Fejiro</t>
+  </si>
+  <si>
+    <t>ADETUBERU Anthony Oluwanifemi</t>
+  </si>
+  <si>
+    <t>FABUSUYI Yetunde Hope</t>
+  </si>
+  <si>
+    <t>TAIWO Temitope Joseph</t>
+  </si>
+  <si>
+    <t>SOLOMON Ajibade Favour</t>
+  </si>
+  <si>
+    <t>OLAYINKA Olalekan Jacob</t>
+  </si>
+  <si>
+    <t>BABAJIDE Oyetunji</t>
+  </si>
+  <si>
+    <t>ATITI Joy Oghenerukevwe Tekena</t>
+  </si>
+  <si>
+    <t>SAMUEL Onyedika Samuel</t>
+  </si>
+  <si>
+    <t>ABIONA Damilola Peace</t>
+  </si>
+  <si>
+    <t>IKUKOYI Dayo Sunday</t>
+  </si>
+  <si>
+    <t>LAAGO Blessing Kabari</t>
+  </si>
+  <si>
+    <t>IKPURI Eyoanwan Olaitan</t>
+  </si>
+  <si>
+    <t>AKINLEYE Onaopemipo Glory</t>
+  </si>
+  <si>
+    <t>ADEEKO Bridget Olufunmilola</t>
+  </si>
+  <si>
+    <t>OMOYOMI Oluwatosin Clinton</t>
+  </si>
+  <si>
+    <t>ENEBELI Chukwudi</t>
+  </si>
+  <si>
     <t>UGWUOKE Rachael Nneoma</t>
   </si>
   <si>
+    <t>ADEOSUN Taiwo</t>
+  </si>
+  <si>
+    <t>APATA Victor Paul</t>
+  </si>
+  <si>
+    <t>AMURO Abiodun Oluwafemi</t>
+  </si>
+  <si>
+    <t>UGOBI Michael Chidiebere</t>
+  </si>
+  <si>
     <t>EWERE Godswork Odion</t>
   </si>
   <si>
-    <t>LAAGO Blessing Kabari</t>
-  </si>
-  <si>
-    <t>BABAJIDE Oyetunji</t>
-  </si>
-  <si>
-    <t>IKUKOYI Dayo Sunday</t>
-  </si>
-  <si>
-    <t>OMBULE Daniel Blessing</t>
-  </si>
-  <si>
-    <t>OMOYOMI Oluwatosin Clinton</t>
-  </si>
-  <si>
-    <t>SAMUEL Onyedika Samuel</t>
-  </si>
-  <si>
-    <t>ATITI Joy Oghenerukevwe Tekena</t>
-  </si>
-  <si>
-    <t>TAIWO Temitope Joseph</t>
-  </si>
-  <si>
-    <t>ADEOSUN Taiwo</t>
-  </si>
-  <si>
-    <t>OGHENEWOGAGA Michael Fejiro</t>
-  </si>
-  <si>
-    <t>OLAYINKA Olalekan Jacob</t>
-  </si>
-  <si>
-    <t>CHUKWUNURU Christian Chidoziem</t>
-  </si>
-  <si>
-    <t>ABIONA Damilola Peace</t>
-  </si>
-  <si>
-    <t>SOLOMON Ajibade Favour</t>
-  </si>
-  <si>
-    <t>FATOBA Ruth Tofunmi</t>
-  </si>
-  <si>
-    <t>OKEOWO Toluwani Elizabeth</t>
-  </si>
-  <si>
-    <t>UGOBI Michael Chidiebere</t>
-  </si>
-  <si>
-    <t>AKINLEYE Onaopemipo Glory</t>
-  </si>
-  <si>
-    <t>ANUKAM Chinazaekpere Peace</t>
-  </si>
-  <si>
-    <t>FABUSUYI Yetunde Hope</t>
-  </si>
-  <si>
-    <t>APATA Victor Paul</t>
-  </si>
-  <si>
     <t>AFOLABI Bukola Adejoke</t>
-  </si>
-  <si>
-    <t>AMENE Ter'Hemen</t>
   </si>
 </sst>
 </file>
@@ -502,7 +523,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -540,7 +561,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -551,10 +572,10 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C6">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -562,10 +583,10 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C7">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -573,7 +594,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -584,7 +605,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C9">
         <v>0</v>
@@ -598,7 +619,7 @@
         <v>3</v>
       </c>
       <c r="C10">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -606,10 +627,10 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C11">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -620,7 +641,7 @@
         <v>2</v>
       </c>
       <c r="C12">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -628,7 +649,7 @@
         <v>13</v>
       </c>
       <c r="B13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C13">
         <v>0</v>
@@ -642,7 +663,7 @@
         <v>4</v>
       </c>
       <c r="C14">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -650,10 +671,10 @@
         <v>15</v>
       </c>
       <c r="B15">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C15">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -661,10 +682,10 @@
         <v>16</v>
       </c>
       <c r="B16">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C16">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -672,10 +693,10 @@
         <v>17</v>
       </c>
       <c r="B17">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C17">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -683,7 +704,7 @@
         <v>18</v>
       </c>
       <c r="B18">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C18">
         <v>0</v>
@@ -694,10 +715,10 @@
         <v>19</v>
       </c>
       <c r="B19">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C19">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -705,7 +726,7 @@
         <v>20</v>
       </c>
       <c r="B20">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C20">
         <v>0</v>
@@ -716,7 +737,7 @@
         <v>21</v>
       </c>
       <c r="B21">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C21">
         <v>0</v>
@@ -738,7 +759,7 @@
         <v>23</v>
       </c>
       <c r="B23">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C23">
         <v>2</v>
@@ -749,7 +770,7 @@
         <v>24</v>
       </c>
       <c r="B24">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C24">
         <v>0</v>
@@ -760,7 +781,7 @@
         <v>25</v>
       </c>
       <c r="B25">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C25">
         <v>0</v>
@@ -771,10 +792,10 @@
         <v>26</v>
       </c>
       <c r="B26">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C26">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -782,10 +803,10 @@
         <v>27</v>
       </c>
       <c r="B27">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C27">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -793,7 +814,7 @@
         <v>28</v>
       </c>
       <c r="B28">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C28">
         <v>0</v>
@@ -804,10 +825,10 @@
         <v>29</v>
       </c>
       <c r="B29">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C29">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -815,9 +836,86 @@
         <v>30</v>
       </c>
       <c r="B30">
+        <v>0</v>
+      </c>
+      <c r="C30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>31</v>
+      </c>
+      <c r="B31">
         <v>1</v>
       </c>
-      <c r="C30">
+      <c r="C31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>32</v>
+      </c>
+      <c r="B32">
+        <v>0</v>
+      </c>
+      <c r="C32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>33</v>
+      </c>
+      <c r="B33">
+        <v>4</v>
+      </c>
+      <c r="C33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>34</v>
+      </c>
+      <c r="B34">
+        <v>0</v>
+      </c>
+      <c r="C34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>35</v>
+      </c>
+      <c r="B35">
+        <v>6</v>
+      </c>
+      <c r="C35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>36</v>
+      </c>
+      <c r="B36">
+        <v>4</v>
+      </c>
+      <c r="C36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>37</v>
+      </c>
+      <c r="B37">
+        <v>1</v>
+      </c>
+      <c r="C37">
         <v>1</v>
       </c>
     </row>

</xml_diff>